<commit_message>
Add Google Sheets version of the schedule with institutional account permissions
- Created README.md for Google Sheets version detailing functionality and user roles.
- Added appsscript.json for Google Apps Script configuration.
- Removed contrasenas.csv for security, transitioning to a permission-based system.
- Updated Excel files for the consolidated schedule and Google Sheets template.
- Implemented scripts to generate Excel and Google Sheets templates, including user instructions and role management.
- Introduced plantillas.py for reading templates and writing program structures.
</commit_message>
<xml_diff>
--- a/salida/Cronograma 2027 Bloque Neón - Consolidado.xlsx
+++ b/salida/Cronograma 2027 Bloque Neón - Consolidado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <workbookProtection workbookPassword="B883" lockStructure="1"/>
+  <workbookProtection workbookPassword="868A" lockStructure="1"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
@@ -835,7 +835,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection password="B883" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="868A" sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -6547,10 +6547,10 @@
       <c r="AF153" s="13"/>
     </row>
   </sheetData>
-  <sheetProtection password="B883" sheet="1" objects="1" scenarios="1" formatColumns="0" formatRows="0" autoFilter="0"/>
+  <sheetProtection password="868A" sheet="1" objects="1" scenarios="1" formatColumns="0" formatRows="0" autoFilter="0"/>
   <protectedRanges>
-    <protectedRange password="B938" sqref="B4:K153 M4:M153 W4:W153" name="Programa_MM"/>
-    <protectedRange password="D73A" sqref="L4:L153 N4:V153 X4:AF153" name="CASA_MM"/>
+    <protectedRange password="D7AF" sqref="B4:K153 M4:M153 W4:W153" name="Programa_MM"/>
+    <protectedRange password="D146" sqref="L4:L153 N4:V153 X4:AF153" name="CASA_MM"/>
   </protectedRanges>
   <autoFilter ref="A3:AF153"/>
   <dataValidations count="10">
@@ -12296,10 +12296,10 @@
       <c r="AF153" s="13"/>
     </row>
   </sheetData>
-  <sheetProtection password="B883" sheet="1" objects="1" scenarios="1" formatColumns="0" formatRows="0" autoFilter="0"/>
+  <sheetProtection password="868A" sheet="1" objects="1" scenarios="1" formatColumns="0" formatRows="0" autoFilter="0"/>
   <protectedRanges>
-    <protectedRange password="C3BF" sqref="B4:K153 M4:M153 W4:W153" name="Programa_MSCM"/>
-    <protectedRange password="D73A" sqref="L4:L153 N4:V153 X4:AF153" name="CASA_MSCM"/>
+    <protectedRange password="9F74" sqref="B4:K153 M4:M153 W4:W153" name="Programa_MSCM"/>
+    <protectedRange password="D146" sqref="L4:L153 N4:V153 X4:AF153" name="CASA_MSCM"/>
   </protectedRanges>
   <autoFilter ref="A3:AF153"/>
   <dataValidations count="10">
@@ -18045,10 +18045,10 @@
       <c r="AF153" s="13"/>
     </row>
   </sheetData>
-  <sheetProtection password="B883" sheet="1" objects="1" scenarios="1" formatColumns="0" formatRows="0" autoFilter="0"/>
+  <sheetProtection password="868A" sheet="1" objects="1" scenarios="1" formatColumns="0" formatRows="0" autoFilter="0"/>
   <protectedRanges>
-    <protectedRange password="C469" sqref="B4:K153 M4:M153 W4:W153" name="Programa_PTMBA"/>
-    <protectedRange password="D73A" sqref="L4:L153 N4:V153 X4:AF153" name="CASA_PTMBA"/>
+    <protectedRange password="8DFF" sqref="B4:K153 M4:M153 W4:W153" name="Programa_PTMBA"/>
+    <protectedRange password="D146" sqref="L4:L153 N4:V153 X4:AF153" name="CASA_PTMBA"/>
   </protectedRanges>
   <autoFilter ref="A3:AF153"/>
   <dataValidations count="10">
@@ -23794,10 +23794,10 @@
       <c r="AF153" s="13"/>
     </row>
   </sheetData>
-  <sheetProtection password="B883" sheet="1" objects="1" scenarios="1" formatColumns="0" formatRows="0" autoFilter="0"/>
+  <sheetProtection password="868A" sheet="1" objects="1" scenarios="1" formatColumns="0" formatRows="0" autoFilter="0"/>
   <protectedRanges>
-    <protectedRange password="B7E1" sqref="B4:K153 M4:M153 W4:W153" name="Programa_Pregrado_CEMS"/>
-    <protectedRange password="D73A" sqref="L4:L153 N4:V153 X4:AF153" name="CASA_Pregrado_CEMS"/>
+    <protectedRange password="BEB4" sqref="B4:K153 M4:M153 W4:W153" name="Programa_Pregrado_CEMS"/>
+    <protectedRange password="D146" sqref="L4:L153 N4:V153 X4:AF153" name="CASA_Pregrado_CEMS"/>
   </protectedRanges>
   <autoFilter ref="A3:AF153"/>
   <dataValidations count="10">
@@ -23987,7 +23987,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection password="B883" sheet="1" objects="1" scenarios="1" formatColumns="0"/>
+  <sheetProtection password="868A" sheet="1" objects="1" scenarios="1" formatColumns="0"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -29699,10 +29699,10 @@
       <c r="AF153" s="13"/>
     </row>
   </sheetData>
-  <sheetProtection password="B883" sheet="1" objects="1" scenarios="1" formatColumns="0" formatRows="0" autoFilter="0"/>
+  <sheetProtection password="868A" sheet="1" objects="1" scenarios="1" formatColumns="0" formatRows="0" autoFilter="0"/>
   <protectedRanges>
-    <protectedRange password="D529" sqref="B4:K153 M4:M153 W4:W153" name="Programa_AFIN"/>
-    <protectedRange password="D73A" sqref="L4:L153 N4:V153 X4:AF153" name="CASA_AFIN"/>
+    <protectedRange password="C368" sqref="B4:K153 M4:M153 W4:W153" name="Programa_AFIN"/>
+    <protectedRange password="D146" sqref="L4:L153 N4:V153 X4:AF153" name="CASA_AFIN"/>
   </protectedRanges>
   <autoFilter ref="A3:AF153"/>
   <dataValidations count="10">
@@ -35448,10 +35448,10 @@
       <c r="AF153" s="13"/>
     </row>
   </sheetData>
-  <sheetProtection password="B883" sheet="1" objects="1" scenarios="1" formatColumns="0" formatRows="0" autoFilter="0"/>
+  <sheetProtection password="868A" sheet="1" objects="1" scenarios="1" formatColumns="0" formatRows="0" autoFilter="0"/>
   <protectedRanges>
-    <protectedRange password="BC6A" sqref="B4:K153 M4:M153 W4:W153" name="Programa_EMBA"/>
-    <protectedRange password="D73A" sqref="L4:L153 N4:V153 X4:AF153" name="CASA_EMBA"/>
+    <protectedRange password="F239" sqref="B4:K153 M4:M153 W4:W153" name="Programa_EMBA"/>
+    <protectedRange password="D146" sqref="L4:L153 N4:V153 X4:AF153" name="CASA_EMBA"/>
   </protectedRanges>
   <autoFilter ref="A3:AF153"/>
   <dataValidations count="10">
@@ -41197,10 +41197,10 @@
       <c r="AF153" s="13"/>
     </row>
   </sheetData>
-  <sheetProtection password="B883" sheet="1" objects="1" scenarios="1" formatColumns="0" formatRows="0" autoFilter="0"/>
+  <sheetProtection password="868A" sheet="1" objects="1" scenarios="1" formatColumns="0" formatRows="0" autoFilter="0"/>
   <protectedRanges>
-    <protectedRange password="A8D6" sqref="B4:K153 M4:M153 W4:W153" name="Programa_IMER"/>
-    <protectedRange password="D73A" sqref="L4:L153 N4:V153 X4:AF153" name="CASA_IMER"/>
+    <protectedRange password="A1BE" sqref="B4:K153 M4:M153 W4:W153" name="Programa_IMER"/>
+    <protectedRange password="D146" sqref="L4:L153 N4:V153 X4:AF153" name="CASA_IMER"/>
   </protectedRanges>
   <autoFilter ref="A3:AF153"/>
   <dataValidations count="10">
@@ -46946,10 +46946,10 @@
       <c r="AF153" s="13"/>
     </row>
   </sheetData>
-  <sheetProtection password="B883" sheet="1" objects="1" scenarios="1" formatColumns="0" formatRows="0" autoFilter="0"/>
+  <sheetProtection password="868A" sheet="1" objects="1" scenarios="1" formatColumns="0" formatRows="0" autoFilter="0"/>
   <protectedRanges>
-    <protectedRange password="DFD1" sqref="B4:K153 M4:M153 W4:W153" name="Programa_MBAOnline"/>
-    <protectedRange password="D73A" sqref="L4:L153 N4:V153 X4:AF153" name="CASA_MBAOnline"/>
+    <protectedRange password="A5B9" sqref="B4:K153 M4:M153 W4:W153" name="Programa_MBAOnline"/>
+    <protectedRange password="D146" sqref="L4:L153 N4:V153 X4:AF153" name="CASA_MBAOnline"/>
   </protectedRanges>
   <autoFilter ref="A3:AF153"/>
   <dataValidations count="10">
@@ -52695,10 +52695,10 @@
       <c r="AF153" s="13"/>
     </row>
   </sheetData>
-  <sheetProtection password="B883" sheet="1" objects="1" scenarios="1" formatColumns="0" formatRows="0" autoFilter="0"/>
+  <sheetProtection password="868A" sheet="1" objects="1" scenarios="1" formatColumns="0" formatRows="0" autoFilter="0"/>
   <protectedRanges>
-    <protectedRange password="C488" sqref="B4:K153 M4:M153 W4:W153" name="Programa_MDP"/>
-    <protectedRange password="D73A" sqref="L4:L153 N4:V153 X4:AF153" name="CASA_MDP"/>
+    <protectedRange password="BDA6" sqref="B4:K153 M4:M153 W4:W153" name="Programa_MDP"/>
+    <protectedRange password="D146" sqref="L4:L153 N4:V153 X4:AF153" name="CASA_MDP"/>
   </protectedRanges>
   <autoFilter ref="A3:AF153"/>
   <dataValidations count="10">
@@ -58444,10 +58444,10 @@
       <c r="AF153" s="13"/>
     </row>
   </sheetData>
-  <sheetProtection password="B883" sheet="1" objects="1" scenarios="1" formatColumns="0" formatRows="0" autoFilter="0"/>
+  <sheetProtection password="868A" sheet="1" objects="1" scenarios="1" formatColumns="0" formatRows="0" autoFilter="0"/>
   <protectedRanges>
-    <protectedRange password="FC8D" sqref="B4:K153 M4:M153 W4:W153" name="Programa_MF"/>
-    <protectedRange password="D73A" sqref="L4:L153 N4:V153 X4:AF153" name="CASA_MF"/>
+    <protectedRange password="8EA8" sqref="B4:K153 M4:M153 W4:W153" name="Programa_MF"/>
+    <protectedRange password="D146" sqref="L4:L153 N4:V153 X4:AF153" name="CASA_MF"/>
   </protectedRanges>
   <autoFilter ref="A3:AF153"/>
   <dataValidations count="10">
@@ -64193,10 +64193,10 @@
       <c r="AF153" s="13"/>
     </row>
   </sheetData>
-  <sheetProtection password="B883" sheet="1" objects="1" scenarios="1" formatColumns="0" formatRows="0" autoFilter="0"/>
+  <sheetProtection password="868A" sheet="1" objects="1" scenarios="1" formatColumns="0" formatRows="0" autoFilter="0"/>
   <protectedRanges>
-    <protectedRange password="B19B" sqref="B4:K153 M4:M153 W4:W153" name="Programa_MGA"/>
-    <protectedRange password="D73A" sqref="L4:L153 N4:V153 X4:AF153" name="CASA_MGA"/>
+    <protectedRange password="9FCE" sqref="B4:K153 M4:M153 W4:W153" name="Programa_MGA"/>
+    <protectedRange password="D146" sqref="L4:L153 N4:V153 X4:AF153" name="CASA_MGA"/>
   </protectedRanges>
   <autoFilter ref="A3:AF153"/>
   <dataValidations count="10">
@@ -69942,10 +69942,10 @@
       <c r="AF153" s="13"/>
     </row>
   </sheetData>
-  <sheetProtection password="B883" sheet="1" objects="1" scenarios="1" formatColumns="0" formatRows="0" autoFilter="0"/>
+  <sheetProtection password="868A" sheet="1" objects="1" scenarios="1" formatColumns="0" formatRows="0" autoFilter="0"/>
   <protectedRanges>
-    <protectedRange password="E771" sqref="B4:K153 M4:M153 W4:W153" name="Programa_MGEST"/>
-    <protectedRange password="D73A" sqref="L4:L153 N4:V153 X4:AF153" name="CASA_MGEST"/>
+    <protectedRange password="9F25" sqref="B4:K153 M4:M153 W4:W153" name="Programa_MGEST"/>
+    <protectedRange password="D146" sqref="L4:L153 N4:V153 X4:AF153" name="CASA_MGEST"/>
   </protectedRanges>
   <autoFilter ref="A3:AF153"/>
   <dataValidations count="10">

</xml_diff>